<commit_message>
dry matter content added
</commit_message>
<xml_diff>
--- a/Results_isofys/tessf.xlsx
+++ b/Results_isofys/tessf.xlsx
@@ -470,7 +470,7 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>[C]%</t>
+          <t>[C]</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
@@ -485,7 +485,7 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>[C_b]%</t>
+          <t>[C_b]</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">

</xml_diff>

<commit_message>
base de datos NUMEX preliminar completa
</commit_message>
<xml_diff>
--- a/Results_isofys/tessf.xlsx
+++ b/Results_isofys/tessf.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH95"/>
+  <dimension ref="A1:AI95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -598,6 +598,11 @@
           <t>specie</t>
         </is>
       </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>Specific leaf area (g/cm²)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
@@ -714,6 +719,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI2" t="n">
+        <v>34.15994277539342</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -830,6 +838,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI3" t="n">
+        <v>33.18294478527607</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
@@ -946,6 +957,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI4" t="n">
+        <v>37.93648208469055</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
@@ -1062,6 +1076,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI5" t="n">
+        <v>40.56470588235294</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
@@ -1178,6 +1195,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI6" t="n">
+        <v>35.25954751131221</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
@@ -1294,6 +1314,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI7" t="n">
+        <v>33.15173383317713</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
@@ -1410,6 +1433,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI8" t="n">
+        <v>30.50483754512636</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
@@ -1526,6 +1552,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI9" t="n">
+        <v>40.07197898423818</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
@@ -1642,6 +1671,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI10" t="n">
+        <v>25.14212910532276</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
@@ -1758,6 +1790,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI11" t="n">
+        <v>34.10823136818687</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
@@ -1874,6 +1909,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI12" t="n">
+        <v>43.40028169014084</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
@@ -1990,6 +2028,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI13" t="n">
+        <v>35.8758865248227</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
@@ -2106,6 +2147,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI14" t="n">
+        <v>31.9693215339233</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
@@ -2222,6 +2266,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI15" t="n">
+        <v>32.25160202360878</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
@@ -2338,6 +2385,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI16" t="n">
+        <v>35.23089668615984</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
@@ -2454,6 +2504,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI17" t="n">
+        <v>34.03149664929263</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
@@ -2570,6 +2623,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI18" t="n">
+        <v>34.42013201320133</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
@@ -2686,6 +2742,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI19" t="n">
+        <v>37.13388601036269</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
@@ -2802,6 +2861,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI20" t="n">
+        <v>34.93205417607223</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
@@ -2918,6 +2980,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI21" t="n">
+        <v>38.12042253521127</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
@@ -3034,6 +3099,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI22" t="n">
+        <v>34.02602230483271</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
@@ -3150,6 +3218,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI23" t="n">
+        <v>36.02815442561206</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
@@ -3266,6 +3337,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI24" t="n">
+        <v>35.10835322195704</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
@@ -3382,6 +3456,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI25" t="n">
+        <v>32.21244286439817</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
@@ -3498,6 +3575,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI26" t="n">
+        <v>38.78301343570058</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
@@ -3614,6 +3694,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI27" t="n">
+        <v>35.49061855670104</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
@@ -3730,6 +3813,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI28" t="n">
+        <v>34.75611814345991</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
@@ -3846,6 +3932,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI29" t="n">
+        <v>34.20469107551487</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
@@ -3962,6 +4051,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI30" t="n">
+        <v>43.41372646184341</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
@@ -4078,6 +4170,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI31" t="n">
+        <v>43.41372646184341</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
@@ -4194,6 +4289,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI32" t="n">
+        <v>38.38884093711468</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
@@ -4310,6 +4408,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI33" t="n">
+        <v>28.00729765590447</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
@@ -4426,6 +4527,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI34" t="n">
+        <v>28.00729765590447</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
@@ -4542,6 +4646,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI35" t="n">
+        <v>37.72970873786407</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
@@ -4658,6 +4765,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI36" t="n">
+        <v>34.93055141579732</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
@@ -4774,6 +4884,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI37" t="n">
+        <v>31.18076158940397</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
@@ -4890,6 +5003,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI38" t="n">
+        <v>41.06741071428572</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
@@ -5006,6 +5122,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI39" t="n">
+        <v>37.32312049433573</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
@@ -5122,6 +5241,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI40" t="n">
+        <v>36.17970168612192</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
@@ -5238,6 +5360,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI41" t="n">
+        <v>32.91402805611222</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
@@ -5354,6 +5479,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI42" t="n">
+        <v>31.10285451197053</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
@@ -5470,6 +5598,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI43" t="n">
+        <v>30.39869888475836</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
@@ -5586,6 +5717,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI44" t="n">
+        <v>37.48323197219809</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
@@ -5702,6 +5836,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI45" t="n">
+        <v>32.09768</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
@@ -5818,6 +5955,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI46" t="n">
+        <v>32.09768</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
@@ -5934,6 +6074,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI47" t="n">
+        <v>39.16065382370111</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
@@ -6050,6 +6193,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI48" t="n">
+        <v>32.11846846846846</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
@@ -6166,6 +6312,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI49" t="n">
+        <v>38.09801840056618</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
@@ -6282,6 +6431,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI50" t="n">
+        <v>37.71034928848641</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
@@ -6398,6 +6550,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI51" t="n">
+        <v>39.72764811490126</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
@@ -6514,6 +6669,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI52" t="n">
+        <v>33.31036454610436</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
@@ -6630,6 +6788,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI53" t="n">
+        <v>34.7460815047022</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
@@ -6746,6 +6907,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI54" t="n">
+        <v>31.98261633011413</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
@@ -6862,6 +7026,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI55" t="n">
+        <v>38.49102196752626</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
@@ -6978,6 +7145,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI56" t="n">
+        <v>35.47107516650809</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
@@ -7094,6 +7264,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI57" t="n">
+        <v>32.22464912280702</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
@@ -7210,6 +7383,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI58" t="n">
+        <v>33.99637952559301</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
@@ -7326,6 +7502,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI59" t="n">
+        <v>33.4044665012407</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
@@ -7442,6 +7621,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI60" t="n">
+        <v>37.73743016759776</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
@@ -7558,6 +7740,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI61" t="n">
+        <v>37.00026553372279</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
@@ -7674,6 +7859,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI62" t="n">
+        <v>45.65359911406424</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
@@ -7790,6 +7978,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI63" t="n">
+        <v>31.62051282051283</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="n">
@@ -7906,6 +8097,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI64" t="n">
+        <v>38.07644376899696</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
@@ -8022,6 +8216,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI65" t="n">
+        <v>34.4926213592233</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="n">
@@ -8138,6 +8335,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI66" t="n">
+        <v>36.54322709163347</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="n">
@@ -8254,6 +8454,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI67" t="n">
+        <v>36.84074074074074</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="n">
@@ -8370,6 +8573,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI68" t="n">
+        <v>36.31700201207244</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="n">
@@ -8486,6 +8692,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI69" t="n">
+        <v>33.07568366592757</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="n">
@@ -8602,6 +8811,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI70" t="n">
+        <v>32.22326111744584</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="n">
@@ -8718,6 +8930,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI71" t="n">
+        <v>36.82448866777225</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="n">
@@ -8832,6 +9047,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI72" t="n">
+        <v>36.82448866777225</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="n">
@@ -8946,6 +9164,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI73" t="n">
+        <v>37.93288288288289</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="n">
@@ -9062,6 +9283,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI74" t="n">
+        <v>39.81607142857143</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="1" t="n">
@@ -9178,6 +9402,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI75" t="n">
+        <v>38.9956570155902</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="1" t="n">
@@ -9294,6 +9521,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI76" t="n">
+        <v>35.01108280254777</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="1" t="n">
@@ -9410,6 +9640,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI77" t="n">
+        <v>35.7625352112676</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="1" t="n">
@@ -9526,6 +9759,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI78" t="n">
+        <v>36.05222437137331</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="1" t="n">
@@ -9642,6 +9878,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI79" t="n">
+        <v>29.2687074829932</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="1" t="n">
@@ -9758,6 +9997,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI80" t="n">
+        <v>40.31574858757062</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="1" t="n">
@@ -9874,6 +10116,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI81" t="n">
+        <v>32.95561719833564</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="1" t="n">
@@ -9990,6 +10235,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI82" t="n">
+        <v>37.79894273127753</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="1" t="n">
@@ -10106,6 +10354,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI83" t="n">
+        <v>31.78387096774194</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="1" t="n">
@@ -10222,6 +10473,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI84" t="n">
+        <v>41.63273092369477</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="1" t="n">
@@ -10338,6 +10592,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI85" t="n">
+        <v>32.12362911266202</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="1" t="n">
@@ -10454,6 +10711,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI86" t="n">
+        <v>39.07777777777778</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="1" t="n">
@@ -10570,6 +10830,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI87" t="n">
+        <v>34.49588744588745</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="1" t="n">
@@ -10686,6 +10949,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI88" t="n">
+        <v>43.50616113744076</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="1" t="n">
@@ -10802,6 +11068,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI89" t="n">
+        <v>41.68621562952244</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="1" t="n">
@@ -10918,6 +11187,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI90" t="n">
+        <v>35.96792650918635</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="1" t="n">
@@ -11034,6 +11306,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI91" t="n">
+        <v>34.36061538461539</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="1" t="n">
@@ -11150,6 +11425,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI92" t="n">
+        <v>35.34196357878068</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="1" t="n">
@@ -11266,6 +11544,9 @@
           <t>lojaensis</t>
         </is>
       </c>
+      <c r="AI93" t="n">
+        <v>38.64987714987715</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="1" t="n">
@@ -11382,6 +11663,9 @@
           <t>sp nov</t>
         </is>
       </c>
+      <c r="AI94" t="n">
+        <v>30.17824074074074</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="1" t="n">
@@ -11493,6 +11777,9 @@
         <is>
           <t>lojaensis</t>
         </is>
+      </c>
+      <c r="AI95" t="n">
+        <v>39.28316008316008</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
mas errores corregidos: water content, sla, etc.
</commit_message>
<xml_diff>
--- a/Results_isofys/tessf.xlsx
+++ b/Results_isofys/tessf.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI95"/>
+  <dimension ref="A1:AH95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -598,11 +598,6 @@
           <t>specie</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
-        <is>
-          <t>Specific leaf area (g/cm²)</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
@@ -719,9 +714,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI2" t="n">
-        <v>34.15994277539342</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -838,9 +830,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI3" t="n">
-        <v>33.18294478527607</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
@@ -957,9 +946,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI4" t="n">
-        <v>37.93648208469055</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
@@ -1076,9 +1062,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI5" t="n">
-        <v>40.56470588235294</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
@@ -1195,9 +1178,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI6" t="n">
-        <v>35.25954751131221</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
@@ -1314,9 +1294,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI7" t="n">
-        <v>33.15173383317713</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
@@ -1433,9 +1410,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI8" t="n">
-        <v>30.50483754512636</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
@@ -1552,9 +1526,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI9" t="n">
-        <v>40.07197898423818</v>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
@@ -1671,9 +1642,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI10" t="n">
-        <v>25.14212910532276</v>
-      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
@@ -1790,9 +1758,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI11" t="n">
-        <v>34.10823136818687</v>
-      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
@@ -1909,9 +1874,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI12" t="n">
-        <v>43.40028169014084</v>
-      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
@@ -2028,9 +1990,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI13" t="n">
-        <v>35.8758865248227</v>
-      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
@@ -2147,9 +2106,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI14" t="n">
-        <v>31.9693215339233</v>
-      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
@@ -2266,9 +2222,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI15" t="n">
-        <v>32.25160202360878</v>
-      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
@@ -2385,9 +2338,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI16" t="n">
-        <v>35.23089668615984</v>
-      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
@@ -2504,9 +2454,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI17" t="n">
-        <v>34.03149664929263</v>
-      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
@@ -2623,9 +2570,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI18" t="n">
-        <v>34.42013201320133</v>
-      </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
@@ -2742,9 +2686,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI19" t="n">
-        <v>37.13388601036269</v>
-      </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
@@ -2861,9 +2802,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI20" t="n">
-        <v>34.93205417607223</v>
-      </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
@@ -2980,9 +2918,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI21" t="n">
-        <v>38.12042253521127</v>
-      </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
@@ -3099,9 +3034,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI22" t="n">
-        <v>34.02602230483271</v>
-      </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
@@ -3218,9 +3150,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI23" t="n">
-        <v>36.02815442561206</v>
-      </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
@@ -3337,9 +3266,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI24" t="n">
-        <v>35.10835322195704</v>
-      </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
@@ -3456,9 +3382,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI25" t="n">
-        <v>32.21244286439817</v>
-      </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
@@ -3575,9 +3498,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI26" t="n">
-        <v>38.78301343570058</v>
-      </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
@@ -3694,9 +3614,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI27" t="n">
-        <v>35.49061855670104</v>
-      </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
@@ -3813,9 +3730,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI28" t="n">
-        <v>34.75611814345991</v>
-      </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
@@ -3932,9 +3846,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI29" t="n">
-        <v>34.20469107551487</v>
-      </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
@@ -4051,9 +3962,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI30" t="n">
-        <v>43.41372646184341</v>
-      </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
@@ -4170,9 +4078,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI31" t="n">
-        <v>43.41372646184341</v>
-      </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
@@ -4289,9 +4194,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI32" t="n">
-        <v>38.38884093711468</v>
-      </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
@@ -4408,9 +4310,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI33" t="n">
-        <v>28.00729765590447</v>
-      </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
@@ -4527,9 +4426,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI34" t="n">
-        <v>28.00729765590447</v>
-      </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
@@ -4646,9 +4542,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI35" t="n">
-        <v>37.72970873786407</v>
-      </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
@@ -4765,9 +4658,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI36" t="n">
-        <v>34.93055141579732</v>
-      </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
@@ -4884,9 +4774,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI37" t="n">
-        <v>31.18076158940397</v>
-      </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
@@ -5003,9 +4890,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI38" t="n">
-        <v>41.06741071428572</v>
-      </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
@@ -5122,9 +5006,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI39" t="n">
-        <v>37.32312049433573</v>
-      </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
@@ -5241,9 +5122,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI40" t="n">
-        <v>36.17970168612192</v>
-      </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
@@ -5360,9 +5238,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI41" t="n">
-        <v>32.91402805611222</v>
-      </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
@@ -5479,9 +5354,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI42" t="n">
-        <v>31.10285451197053</v>
-      </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
@@ -5598,9 +5470,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI43" t="n">
-        <v>30.39869888475836</v>
-      </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
@@ -5717,9 +5586,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI44" t="n">
-        <v>37.48323197219809</v>
-      </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
@@ -5836,9 +5702,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI45" t="n">
-        <v>32.09768</v>
-      </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
@@ -5955,9 +5818,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI46" t="n">
-        <v>32.09768</v>
-      </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
@@ -6074,9 +5934,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI47" t="n">
-        <v>39.16065382370111</v>
-      </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
@@ -6193,9 +6050,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI48" t="n">
-        <v>32.11846846846846</v>
-      </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
@@ -6312,9 +6166,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI49" t="n">
-        <v>38.09801840056618</v>
-      </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
@@ -6431,9 +6282,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI50" t="n">
-        <v>37.71034928848641</v>
-      </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
@@ -6550,9 +6398,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI51" t="n">
-        <v>39.72764811490126</v>
-      </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
@@ -6669,9 +6514,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI52" t="n">
-        <v>33.31036454610436</v>
-      </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
@@ -6788,9 +6630,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI53" t="n">
-        <v>34.7460815047022</v>
-      </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
@@ -6907,9 +6746,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI54" t="n">
-        <v>31.98261633011413</v>
-      </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
@@ -7026,9 +6862,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI55" t="n">
-        <v>38.49102196752626</v>
-      </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
@@ -7145,9 +6978,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI56" t="n">
-        <v>35.47107516650809</v>
-      </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
@@ -7264,9 +7094,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI57" t="n">
-        <v>32.22464912280702</v>
-      </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
@@ -7383,9 +7210,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI58" t="n">
-        <v>33.99637952559301</v>
-      </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
@@ -7502,9 +7326,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI59" t="n">
-        <v>33.4044665012407</v>
-      </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
@@ -7621,9 +7442,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI60" t="n">
-        <v>37.73743016759776</v>
-      </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
@@ -7740,9 +7558,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI61" t="n">
-        <v>37.00026553372279</v>
-      </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
@@ -7859,9 +7674,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI62" t="n">
-        <v>45.65359911406424</v>
-      </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
@@ -7978,9 +7790,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI63" t="n">
-        <v>31.62051282051283</v>
-      </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="n">
@@ -8097,9 +7906,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI64" t="n">
-        <v>38.07644376899696</v>
-      </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
@@ -8216,9 +8022,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI65" t="n">
-        <v>34.4926213592233</v>
-      </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="n">
@@ -8335,9 +8138,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI66" t="n">
-        <v>36.54322709163347</v>
-      </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="n">
@@ -8454,9 +8254,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI67" t="n">
-        <v>36.84074074074074</v>
-      </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="n">
@@ -8573,9 +8370,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI68" t="n">
-        <v>36.31700201207244</v>
-      </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="n">
@@ -8692,9 +8486,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI69" t="n">
-        <v>33.07568366592757</v>
-      </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="n">
@@ -8811,9 +8602,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI70" t="n">
-        <v>32.22326111744584</v>
-      </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="n">
@@ -8930,9 +8718,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI71" t="n">
-        <v>36.82448866777225</v>
-      </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="n">
@@ -9047,9 +8832,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI72" t="n">
-        <v>36.82448866777225</v>
-      </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="n">
@@ -9164,9 +8946,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI73" t="n">
-        <v>37.93288288288289</v>
-      </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="n">
@@ -9283,9 +9062,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI74" t="n">
-        <v>39.81607142857143</v>
-      </c>
     </row>
     <row r="75">
       <c r="A75" s="1" t="n">
@@ -9402,9 +9178,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI75" t="n">
-        <v>38.9956570155902</v>
-      </c>
     </row>
     <row r="76">
       <c r="A76" s="1" t="n">
@@ -9521,9 +9294,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI76" t="n">
-        <v>35.01108280254777</v>
-      </c>
     </row>
     <row r="77">
       <c r="A77" s="1" t="n">
@@ -9640,9 +9410,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI77" t="n">
-        <v>35.7625352112676</v>
-      </c>
     </row>
     <row r="78">
       <c r="A78" s="1" t="n">
@@ -9759,9 +9526,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI78" t="n">
-        <v>36.05222437137331</v>
-      </c>
     </row>
     <row r="79">
       <c r="A79" s="1" t="n">
@@ -9878,9 +9642,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI79" t="n">
-        <v>29.2687074829932</v>
-      </c>
     </row>
     <row r="80">
       <c r="A80" s="1" t="n">
@@ -9997,9 +9758,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI80" t="n">
-        <v>40.31574858757062</v>
-      </c>
     </row>
     <row r="81">
       <c r="A81" s="1" t="n">
@@ -10116,9 +9874,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI81" t="n">
-        <v>32.95561719833564</v>
-      </c>
     </row>
     <row r="82">
       <c r="A82" s="1" t="n">
@@ -10235,9 +9990,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI82" t="n">
-        <v>37.79894273127753</v>
-      </c>
     </row>
     <row r="83">
       <c r="A83" s="1" t="n">
@@ -10354,9 +10106,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI83" t="n">
-        <v>31.78387096774194</v>
-      </c>
     </row>
     <row r="84">
       <c r="A84" s="1" t="n">
@@ -10473,9 +10222,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI84" t="n">
-        <v>41.63273092369477</v>
-      </c>
     </row>
     <row r="85">
       <c r="A85" s="1" t="n">
@@ -10592,9 +10338,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI85" t="n">
-        <v>32.12362911266202</v>
-      </c>
     </row>
     <row r="86">
       <c r="A86" s="1" t="n">
@@ -10711,9 +10454,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI86" t="n">
-        <v>39.07777777777778</v>
-      </c>
     </row>
     <row r="87">
       <c r="A87" s="1" t="n">
@@ -10830,9 +10570,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI87" t="n">
-        <v>34.49588744588745</v>
-      </c>
     </row>
     <row r="88">
       <c r="A88" s="1" t="n">
@@ -10949,9 +10686,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI88" t="n">
-        <v>43.50616113744076</v>
-      </c>
     </row>
     <row r="89">
       <c r="A89" s="1" t="n">
@@ -11068,9 +10802,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI89" t="n">
-        <v>41.68621562952244</v>
-      </c>
     </row>
     <row r="90">
       <c r="A90" s="1" t="n">
@@ -11187,9 +10918,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI90" t="n">
-        <v>35.96792650918635</v>
-      </c>
     </row>
     <row r="91">
       <c r="A91" s="1" t="n">
@@ -11306,9 +11034,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI91" t="n">
-        <v>34.36061538461539</v>
-      </c>
     </row>
     <row r="92">
       <c r="A92" s="1" t="n">
@@ -11425,9 +11150,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI92" t="n">
-        <v>35.34196357878068</v>
-      </c>
     </row>
     <row r="93">
       <c r="A93" s="1" t="n">
@@ -11544,9 +11266,6 @@
           <t>lojaensis</t>
         </is>
       </c>
-      <c r="AI93" t="n">
-        <v>38.64987714987715</v>
-      </c>
     </row>
     <row r="94">
       <c r="A94" s="1" t="n">
@@ -11663,9 +11382,6 @@
           <t>sp nov</t>
         </is>
       </c>
-      <c r="AI94" t="n">
-        <v>30.17824074074074</v>
-      </c>
     </row>
     <row r="95">
       <c r="A95" s="1" t="n">
@@ -11777,9 +11493,6 @@
         <is>
           <t>lojaensis</t>
         </is>
-      </c>
-      <c r="AI95" t="n">
-        <v>39.28316008316008</v>
       </c>
     </row>
   </sheetData>

</xml_diff>